<commit_message>
Explication de chaque tag : motifs dans les règles, provenance par objet, API explain, lecture unitaire
- champ motif: sur 31 règles, restitué par RuleSet.explain() et dans la table
  de correspondance
- table provenance (attributs BD Topo consultés, compressés) alimentée par les
  deux moteurs
- /api/bdfrance/explain/{type}/{id} ; le bouton (i) d'iD antépose l'explication
  à la référence OSM
- lecture unitaire /{type}/{id}.json, /full.json, /relations.json, multi-fetch
- base de démo Poitiers reconvertie avec provenance

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/mapping.xlsx
+++ b/docs/mapping.xlsx
@@ -1395,7 +1395,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>branche 7 — exclusif, première correspondance</t>
+          <t>branche 7 — exclusif, première correspondance ; motif : OSM n'a pas de valeur consensuelle pour ces lieux-dits bâtis, et la source ne dit pas s'il s'agit d'un moulin à vent ou à eau : on reste sur le toponyme, nature conservée.</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : « Lieu-dit habité » : `importance` est le seul critère de hiérarchie disponible. Calibration à relire : elle décide de ce qui s'affiche comme village ou comme écart.</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : « Lieu-dit habité » : `importance` est le seul critère de hiérarchie disponible. Calibration à relire : elle décide de ce qui s'affiche comme village ou comme écart.</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : « Lieu-dit habité » : `importance` est le seul critère de hiérarchie disponible. Calibration à relire : elle décide de ce qui s'affiche comme village ou comme écart.</t>
         </is>
       </c>
     </row>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : « Lieu-dit habité » : `importance` est le seul critère de hiérarchie disponible. Calibration à relire : elle décide de ce qui s'affiche comme village ou comme écart.</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : « Lieu-dit habité » : `importance` est le seul critère de hiérarchie disponible. Calibration à relire : elle décide de ce qui s'affiche comme village ou comme écart.</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : « Lieu-dit habité » : `importance` est le seul critère de hiérarchie disponible. Calibration à relire : elle décide de ce qui s'affiche comme village ou comme écart.</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : « Lieu-dit habité » : `importance` est le seul critère de hiérarchie disponible. Calibration à relire : elle décide de ce qui s'affiche comme village ou comme écart.</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : `caravan_site` est l'usage OSM français pour ces aires, malgré l'ambiguïté du terme touristique.</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : `caravan_site` est l'usage OSM français pour ces aires, malgré l'ambiguïté du terme touristique.</t>
         </is>
       </c>
     </row>
@@ -4354,7 +4354,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>branche 59 — exclusif, première correspondance</t>
+          <t>branche 59 — exclusif, première correspondance ; motif : En milieu rural ces salles sont le plus souvent des salles des fêtes : `community_centre` plutôt que `theatre`.</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4435,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>branche 62 — exclusif, première correspondance</t>
+          <t>branche 62 — exclusif, première correspondance ; motif : Nature sans correspondance OSM assumée : `fixme` est un vrai tag, lu par les éditeurs et les outils de contrôle — préférable à un `tourism=attraction` posé au jugé.</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>branche 7 — exclusif, première correspondance</t>
+          <t>branche 7 — exclusif, première correspondance ; motif : 739 entités, toutes « Borne de rechargement électrique » d'après `nature_detaillee` ; la source Etalab (opérateurs IRVE) le confirme.</t>
         </is>
       </c>
     </row>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>branche 7 — exclusif, première correspondance</t>
+          <t>branche 7 — exclusif, première correspondance ; motif : 739 entités, toutes « Borne de rechargement électrique » d'après `nature_detaillee` ; la source Etalab (opérateurs IRVE) le confirme.</t>
         </is>
       </c>
     </row>
@@ -7807,7 +7807,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>branche 1 — exclusif, première correspondance</t>
+          <t>branche 1 — exclusif, première correspondance ; motif : Réservoir surélevé : `man_made=water_tower` ; c'est aussi un bâtiment.</t>
         </is>
       </c>
     </row>
@@ -7834,7 +7834,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>branche 1 — exclusif, première correspondance</t>
+          <t>branche 1 — exclusif, première correspondance ; motif : Réservoir surélevé : `man_made=water_tower` ; c'est aussi un bâtiment.</t>
         </is>
       </c>
     </row>
@@ -12159,7 +12159,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>branche 1 — exclusif, première correspondance</t>
+          <t>branche 1 — exclusif, première correspondance ; motif : La restriction décrit ce qu'EST la voie — un aménagement cyclable propre — pas une contrainte qui s'y ajoute. Elle prime donc sur la nature.</t>
         </is>
       </c>
     </row>
@@ -12321,7 +12321,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>branche 6 — exclusif, première correspondance</t>
+          <t>branche 6 — exclusif, première correspondance ; motif : « Chemin » BD Topo : prévu pour les véhicules ou engins d'exploitation, pas forcément carrossable par tous les temps — c'est la définition d'un `track`.</t>
         </is>
       </c>
     </row>
@@ -12348,7 +12348,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>branche 6 — exclusif, première correspondance</t>
+          <t>branche 6 — exclusif, première correspondance ; motif : « Chemin » BD Topo : prévu pour les véhicules ou engins d'exploitation, pas forcément carrossable par tous les temps — c'est la définition d'un `track`.</t>
         </is>
       </c>
     </row>
@@ -12375,7 +12375,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>branche 7 — exclusif, première correspondance</t>
+          <t>branche 7 — exclusif, première correspondance ; motif : Carrossable et publique selon la source (13 privées sur 56 369 dans la Vienne, 54 502 en accès libre) : donc `unclassified`, pas `track`, qui sous-entendrait un usage agricole non établi. Le revêtement est porté par `surface`, requalifiable.</t>
         </is>
       </c>
     </row>
@@ -12402,7 +12402,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>branche 7 — exclusif, première correspondance</t>
+          <t>branche 7 — exclusif, première correspondance ; motif : Carrossable et publique selon la source (13 privées sur 56 369 dans la Vienne, 54 502 en accès libre) : donc `unclassified`, pas `track`, qui sous-entendrait un usage agricole non établi. Le revêtement est porté par `surface`, requalifiable.</t>
         </is>
       </c>
     </row>
@@ -12429,7 +12429,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance ; si nature = Bretelle</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : La BD Topo ne dit pas quelle route la bretelle raccorde ; la classe est déduite de `importance`. IGN affecte à une bretelle « l'importance la moins importante des deux tronçons qu'elle joint ». Approximation à remplacer par une propagation depuis les tronçons connectés. ; si nature = Bretelle</t>
         </is>
       </c>
     </row>
@@ -12456,7 +12456,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance ; si nature = Bretelle</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : La BD Topo ne dit pas quelle route la bretelle raccorde ; la classe est déduite de `importance`. IGN affecte à une bretelle « l'importance la moins importante des deux tronçons qu'elle joint ». Approximation à remplacer par une propagation depuis les tronçons connectés. ; si nature = Bretelle</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance ; si nature = Bretelle</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : La BD Topo ne dit pas quelle route la bretelle raccorde ; la classe est déduite de `importance`. IGN affecte à une bretelle « l'importance la moins importante des deux tronçons qu'elle joint ». Approximation à remplacer par une propagation depuis les tronçons connectés. ; si nature = Bretelle</t>
         </is>
       </c>
     </row>
@@ -12510,7 +12510,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance ; si nature = Bretelle</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : La BD Topo ne dit pas quelle route la bretelle raccorde ; la classe est déduite de `importance`. IGN affecte à une bretelle « l'importance la moins importante des deux tronçons qu'elle joint ». Approximation à remplacer par une propagation depuis les tronçons connectés. ; si nature = Bretelle</t>
         </is>
       </c>
     </row>
@@ -12537,7 +12537,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance ; si nature = Bretelle</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : La BD Topo ne dit pas quelle route la bretelle raccorde ; la classe est déduite de `importance`. IGN affecte à une bretelle « l'importance la moins importante des deux tronçons qu'elle joint ». Approximation à remplacer par une propagation depuis les tronçons connectés. ; si nature = Bretelle</t>
         </is>
       </c>
     </row>
@@ -12564,7 +12564,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance ; si nature = Bretelle</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : La BD Topo ne dit pas quelle route la bretelle raccorde ; la classe est déduite de `importance`. IGN affecte à une bretelle « l'importance la moins importante des deux tronçons qu'elle joint ». Approximation à remplacer par une propagation depuis les tronçons connectés. ; si nature = Bretelle</t>
         </is>
       </c>
     </row>
@@ -12591,7 +12591,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>branche 8 — exclusif, première correspondance ; si nature = Bretelle</t>
+          <t>branche 8 — exclusif, première correspondance ; motif : La BD Topo ne dit pas quelle route la bretelle raccorde ; la classe est déduite de `importance`. IGN affecte à une bretelle « l'importance la moins importante des deux tronçons qu'elle joint ». Approximation à remplacer par une propagation depuis les tronçons connectés. ; si nature = Bretelle</t>
         </is>
       </c>
     </row>
@@ -12618,7 +12618,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : `junction=roundabout` est une forme, pas une classe : la classe vient de `importance`, à défaut de connaître la route la plus importante qui aboutit à l'anneau.</t>
         </is>
       </c>
     </row>
@@ -12645,7 +12645,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : `junction=roundabout` est une forme, pas une classe : la classe vient de `importance`, à défaut de connaître la route la plus importante qui aboutit à l'anneau.</t>
         </is>
       </c>
     </row>
@@ -12672,7 +12672,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance ; si nature = Rond-point</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : `junction=roundabout` est une forme, pas une classe : la classe vient de `importance`, à défaut de connaître la route la plus importante qui aboutit à l'anneau. ; si nature = Rond-point</t>
         </is>
       </c>
     </row>
@@ -12699,7 +12699,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance ; si nature = Rond-point</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : `junction=roundabout` est une forme, pas une classe : la classe vient de `importance`, à défaut de connaître la route la plus importante qui aboutit à l'anneau. ; si nature = Rond-point</t>
         </is>
       </c>
     </row>
@@ -12726,7 +12726,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance ; si nature = Rond-point</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : `junction=roundabout` est une forme, pas une classe : la classe vient de `importance`, à défaut de connaître la route la plus importante qui aboutit à l'anneau. ; si nature = Rond-point</t>
         </is>
       </c>
     </row>
@@ -12753,7 +12753,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance ; si nature = Rond-point</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : `junction=roundabout` est une forme, pas une classe : la classe vient de `importance`, à défaut de connaître la route la plus importante qui aboutit à l'anneau. ; si nature = Rond-point</t>
         </is>
       </c>
     </row>
@@ -12780,7 +12780,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance ; si nature = Rond-point</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : `junction=roundabout` est une forme, pas une classe : la classe vient de `importance`, à défaut de connaître la route la plus importante qui aboutit à l'anneau. ; si nature = Rond-point</t>
         </is>
       </c>
     </row>
@@ -12807,7 +12807,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance ; si nature = Rond-point</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : `junction=roundabout` est une forme, pas une classe : la classe vient de `importance`, à défaut de connaître la route la plus importante qui aboutit à l'anneau. ; si nature = Rond-point</t>
         </is>
       </c>
     </row>
@@ -12834,7 +12834,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance ; si nature = Rond-point</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : `junction=roundabout` est une forme, pas une classe : la classe vient de `importance`, à défaut de connaître la route la plus importante qui aboutit à l'anneau. ; si nature = Rond-point</t>
         </is>
       </c>
     </row>
@@ -12861,7 +12861,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>branche 10 — exclusif, première correspondance</t>
+          <t>branche 10 — exclusif, première correspondance ; motif : Le classement administratif fait autorité quand il est renseigné (15,7 % des tronçons de la Vienne).</t>
         </is>
       </c>
     </row>
@@ -12942,7 +12942,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>branche 13 — exclusif, première correspondance ; si cpx_classement_administratif contient « Départementale »</t>
+          <t>branche 13 — exclusif, première correspondance ; motif : Départementale : la classe suit `importance`, qu'IGN définit comme une hiérarchisation fonctionnelle du réseau (non administrative). Mesuré : importance 4 = 29 790 D sur 34 022 tronçons. ; si cpx_classement_administratif contient « Départementale »</t>
         </is>
       </c>
     </row>
@@ -12969,7 +12969,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>branche 13 — exclusif, première correspondance ; si cpx_classement_administratif contient « Départementale »</t>
+          <t>branche 13 — exclusif, première correspondance ; motif : Départementale : la classe suit `importance`, qu'IGN définit comme une hiérarchisation fonctionnelle du réseau (non administrative). Mesuré : importance 4 = 29 790 D sur 34 022 tronçons. ; si cpx_classement_administratif contient « Départementale »</t>
         </is>
       </c>
     </row>
@@ -12996,7 +12996,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>branche 13 — exclusif, première correspondance ; si cpx_classement_administratif contient « Départementale »</t>
+          <t>branche 13 — exclusif, première correspondance ; motif : Départementale : la classe suit `importance`, qu'IGN définit comme une hiérarchisation fonctionnelle du réseau (non administrative). Mesuré : importance 4 = 29 790 D sur 34 022 tronçons. ; si cpx_classement_administratif contient « Départementale »</t>
         </is>
       </c>
     </row>
@@ -13023,7 +13023,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>branche 13 — exclusif, première correspondance ; si cpx_classement_administratif contient « Départementale »</t>
+          <t>branche 13 — exclusif, première correspondance ; motif : Départementale : la classe suit `importance`, qu'IGN définit comme une hiérarchisation fonctionnelle du réseau (non administrative). Mesuré : importance 4 = 29 790 D sur 34 022 tronçons. ; si cpx_classement_administratif contient « Départementale »</t>
         </is>
       </c>
     </row>
@@ -13050,7 +13050,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>branche 13 — exclusif, première correspondance ; si cpx_classement_administratif contient « Départementale »</t>
+          <t>branche 13 — exclusif, première correspondance ; motif : Départementale : la classe suit `importance`, qu'IGN définit comme une hiérarchisation fonctionnelle du réseau (non administrative). Mesuré : importance 4 = 29 790 D sur 34 022 tronçons. ; si cpx_classement_administratif contient « Départementale »</t>
         </is>
       </c>
     </row>
@@ -13077,7 +13077,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>branche 13 — exclusif, première correspondance ; si cpx_classement_administratif contient « Départementale »</t>
+          <t>branche 13 — exclusif, première correspondance ; motif : Départementale : la classe suit `importance`, qu'IGN définit comme une hiérarchisation fonctionnelle du réseau (non administrative). Mesuré : importance 4 = 29 790 D sur 34 022 tronçons. ; si cpx_classement_administratif contient « Départementale »</t>
         </is>
       </c>
     </row>
@@ -13104,7 +13104,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>branche 13 — exclusif, première correspondance ; si cpx_classement_administratif contient « Départementale »</t>
+          <t>branche 13 — exclusif, première correspondance ; motif : Départementale : la classe suit `importance`, qu'IGN définit comme une hiérarchisation fonctionnelle du réseau (non administrative). Mesuré : importance 4 = 29 790 D sur 34 022 tronçons. ; si cpx_classement_administratif contient « Départementale »</t>
         </is>
       </c>
     </row>
@@ -13131,7 +13131,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>branche 14 — exclusif, première correspondance</t>
+          <t>branche 14 — exclusif, première correspondance ; motif : Type autoroutier sans classement Autoroute : le préfixe du numéro tranche (A10 → motorway ; N147 en voie express → trunk).</t>
         </is>
       </c>
     </row>
@@ -13374,7 +13374,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>branche 17 — exclusif, première correspondance</t>
+          <t>branche 17 — exclusif, première correspondance ; motif : Importance 5 = desserte locale (129 135 tronçons, le gros du réseau). `urbain` sépare la voirie de lotissement (`residential`) de la voie communale rase-campagne (`unclassified`).</t>
         </is>
       </c>
     </row>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance ; si nature = Route à 1 chaussée</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : Repli nature × importance pour les 84,3 % de tronçons sans classement administratif. ; si nature = Route à 1 chaussée</t>
         </is>
       </c>
     </row>
@@ -13428,7 +13428,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance ; si nature = Route à 1 chaussée</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : Repli nature × importance pour les 84,3 % de tronçons sans classement administratif. ; si nature = Route à 1 chaussée</t>
         </is>
       </c>
     </row>
@@ -13455,7 +13455,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance ; si nature = Route à 1 chaussée</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : Repli nature × importance pour les 84,3 % de tronçons sans classement administratif. ; si nature = Route à 1 chaussée</t>
         </is>
       </c>
     </row>
@@ -13482,7 +13482,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance ; si nature = Route à 1 chaussée</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : Repli nature × importance pour les 84,3 % de tronçons sans classement administratif. ; si nature = Route à 1 chaussée</t>
         </is>
       </c>
     </row>
@@ -13509,7 +13509,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance ; si nature = Route à 1 chaussée</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : Repli nature × importance pour les 84,3 % de tronçons sans classement administratif. ; si nature = Route à 1 chaussée</t>
         </is>
       </c>
     </row>
@@ -13536,7 +13536,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance ; si nature = Route à 1 chaussée</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : Repli nature × importance pour les 84,3 % de tronçons sans classement administratif. ; si nature = Route à 1 chaussée</t>
         </is>
       </c>
     </row>
@@ -13563,7 +13563,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance ; si nature = Route à 1 chaussée</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : Repli nature × importance pour les 84,3 % de tronçons sans classement administratif. ; si nature = Route à 1 chaussée</t>
         </is>
       </c>
     </row>
@@ -17068,7 +17068,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>branche 2 — exclusif, première correspondance</t>
+          <t>branche 2 — exclusif, première correspondance ; motif : Un bois nommé reste un toponyme : son emprise, quand elle existe, est portée par `zone_de_vegetation`. `natural=wood` sur un point dupliquerait l'information.</t>
         </is>
       </c>
     </row>
@@ -20274,7 +20274,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>branche 1 — exclusif, première correspondance</t>
+          <t>branche 1 — exclusif, première correspondance ; motif : Un fossé reste un fossé quelle que soit sa largeur : la nature de l'ouvrage l'emporte sur la classe dimensionnelle.</t>
         </is>
       </c>
     </row>
@@ -20382,7 +20382,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>branche 4 — exclusif, première correspondance</t>
+          <t>branche 4 — exclusif, première correspondance ; motif : `classe_de_largeur` est le seul critère dimensionnel disponible ; le seuil OSM usuel entre `stream` et `river` (≈ 5 m) tombe exactement sur une borne de la nomenclature IGN.</t>
         </is>
       </c>
     </row>
@@ -20434,7 +20434,11 @@
           <t>culvert</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>motif : Écoulement busé sous un remblai ou une voirie : `tunnel=culvert`.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -20457,7 +20461,11 @@
           <t>-1</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>motif : Écoulement busé sous un remblai ou une voirie : `tunnel=culvert`.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -25254,7 +25262,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>branche 14 — exclusif, première correspondance</t>
+          <t>branche 14 — exclusif, première correspondance ; motif : 229 978 bâtiments résidentiels à exactement 1 logement dans la Vienne : `nombre_de_logements` étaye solidement la distinction maison / immeuble.</t>
         </is>
       </c>
     </row>
@@ -25281,7 +25289,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>branche 15 — exclusif, première correspondance</t>
+          <t>branche 15 — exclusif, première correspondance ; motif : Plusieurs logements dans un bâtiment résidentiel : immeuble.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25343,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>branche 17 — exclusif, première correspondance</t>
+          <t>branche 17 — exclusif, première correspondance ; motif : OSM n'a pas de valeur consensuelle pour « annexe » (garages, remises, abris confondus) ; `construction_legere` isole au moins les abris légers.</t>
         </is>
       </c>
     </row>
@@ -25362,7 +25370,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>branche 18 — exclusif, première correspondance</t>
+          <t>branche 18 — exclusif, première correspondance ; motif : Annexe sans autre précision : `building=yes` avec l'usage source conservé, plutôt qu'une valeur inventée.</t>
         </is>
       </c>
     </row>
@@ -25524,7 +25532,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>branche 24 — exclusif, première correspondance</t>
+          <t>branche 24 — exclusif, première correspondance ; motif : La nature exclut le résidentiel mais ne tranche pas entre trois fonctions aux valeurs OSM distinctes : en choisir une serait fabriquer de l'information. La nature source est conservée, requalifiable.</t>
         </is>
       </c>
     </row>
@@ -25558,12 +25566,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>nature, usage_1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>(nature ∈ {Eglise, Chapelle}) et (usage_1 = Religieux)</t>
+          <t>(toujours)</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -25576,17 +25584,21 @@
           <t>place_of_worship</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>motif : `nature` donne la forme du bâtiment, `usage_1` atteste l'usage courant : c'est leur conjonction qui justifie `amenity=place_of_worship`, pas la forme seule. all_of: - {nature: [Eglise, Chapelle]} - {usage_1: Religieux}</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>nature, usage_1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>(nature ∈ {Eglise, Chapelle}) et (usage_1 = Religieux)</t>
+          <t>(toujours)</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -25599,7 +25611,11 @@
           <t>christian</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>motif : `nature` donne la forme du bâtiment, `usage_1` atteste l'usage courant : c'est leur conjonction qui justifie `amenity=place_of_worship`, pas la forme seule. all_of: - {nature: [Eglise, Chapelle]} - {usage_1: Religieux}</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -28543,7 +28559,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>branche 3 — exclusif, première correspondance</t>
+          <t>branche 3 — exclusif, première correspondance ; motif : Plantation exploitée : `landuse=forest` plutôt que `natural=wood`, qui suggère un boisement spontané.</t>
         </is>
       </c>
     </row>
@@ -28570,7 +28586,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>branche 3 — exclusif, première correspondance</t>
+          <t>branche 3 — exclusif, première correspondance ; motif : Plantation exploitée : `landuse=forest` plutôt que `natural=wood`, qui suggère un boisement spontané.</t>
         </is>
       </c>
     </row>
@@ -28624,7 +28640,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>branche 5 — exclusif, première correspondance</t>
+          <t>branche 5 — exclusif, première correspondance ; motif : Couvert discontinu, plus proche du fourré que du bois.</t>
         </is>
       </c>
     </row>
@@ -29534,7 +29550,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>branche 5 — exclusif, première correspondance</t>
+          <t>branche 5 — exclusif, première correspondance ; motif : Bassin technique : `landuse=basin` décrit l'ouvrage, `natural=water` décrirait l'eau — ici c'est l'ouvrage qui est cartographié.</t>
         </is>
       </c>
     </row>
@@ -29561,7 +29577,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>branche 5 — exclusif, première correspondance</t>
+          <t>branche 5 — exclusif, première correspondance ; motif : Bassin technique : `landuse=basin` décrit l'ouvrage, `natural=water` décrirait l'eau — ici c'est l'ouvrage qui est cartographié.</t>
         </is>
       </c>
     </row>
@@ -29723,7 +29739,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : « Retenue » (15 876) et « Mare » (7 057) forment l'essentiel du bocage poitevin : petites pièces d'eau, très majoritairement artificielles.</t>
         </is>
       </c>
     </row>
@@ -29750,7 +29766,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>branche 9 — exclusif, première correspondance</t>
+          <t>branche 9 — exclusif, première correspondance ; motif : « Retenue » (15 876) et « Mare » (7 057) forment l'essentiel du bocage poitevin : petites pièces d'eau, très majoritairement artificielles.</t>
         </is>
       </c>
     </row>

</xml_diff>